<commit_message>
Part Selection doc updated. Added source selector, power switch and barrel connector.
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Part Selection.xlsx
+++ b/Documents/Dev-Files/Part Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A2A760E-9BEA-44E8-B0DD-7D29CA73EEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA60CF3-4E79-41AB-98F5-2CD0F47C0470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Component</t>
   </si>
@@ -82,17 +82,47 @@
     <t>DigiKey Alternate</t>
   </si>
   <si>
-    <t>AP2411MP-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> available on both sites but expensive</t>
+    <t>SLG7NT402V</t>
+  </si>
+  <si>
+    <t>Available on sites other than LCSC</t>
+  </si>
+  <si>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>DC-C300-5.5A-2.5</t>
+  </si>
+  <si>
+    <t>TPS2115ADRBTG4</t>
+  </si>
+  <si>
+    <t>Worldway</t>
+  </si>
+  <si>
+    <t>Also available on Aliexpress and chipfind</t>
+  </si>
+  <si>
+    <t>2A Source Selector</t>
+  </si>
+  <si>
+    <t>4A Power switch</t>
+  </si>
+  <si>
+    <t>Ics</t>
+  </si>
+  <si>
+    <t>5.5A Jack DCPowerReceptacle 6.0mm 2.5mm</t>
+  </si>
+  <si>
+    <t>Connector</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,16 +138,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -125,17 +181,148 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -460,98 +647,167 @@
     <col min="3" max="3" width="40.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.42578125" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    <row r="3" spans="1:8" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="B3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="2" t="s">
+      <c r="F3" s="5"/>
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1" t="s">
+    <row r="4" spans="1:8" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8">
+        <v>2</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="2" t="s">
+      <c r="F4" s="9"/>
+      <c r="G4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1" t="s">
+    <row r="5" spans="1:8" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="C5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1" t="s">
+      <c r="F5" s="12"/>
+      <c r="G5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="14" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
+        <v>4</v>
+      </c>
+      <c r="B6" s="16"/>
+      <c r="C6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" s="9"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D13" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:B7"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" xr:uid="{B9773254-489E-4981-AD57-E06C75AC1D1B}"/>
     <hyperlink ref="G3" r:id="rId2" xr:uid="{E9B95C05-B41C-4877-99DA-9D0B95A29B4E}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{2CC3C96D-9B1A-4A63-8F2F-202DB24A48FE}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{7E117F9F-8F90-4E69-A531-92FE100C33C9}"/>
+    <hyperlink ref="G8" r:id="rId5" xr:uid="{0D1B945F-FB9A-413C-807D-F04C4AB6F79F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Client Original BOM and some modification done in Part Selection Sheet
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Part Selection.xlsx
+++ b/Documents/Dev-Files/Part Selection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24620"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA60CF3-4E79-41AB-98F5-2CD0F47C0470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF25AFE-F4FD-48EC-A690-67773A2FFDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,27 +34,15 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>Sr.No</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
     <t>Link</t>
   </si>
   <si>
-    <t>Remark</t>
-  </si>
-  <si>
     <t>LCSC</t>
   </si>
   <si>
-    <t>Manufacturer Part num</t>
-  </si>
-  <si>
     <t>SDB628</t>
   </si>
   <si>
@@ -79,9 +67,6 @@
     <t>Alternate IC available on both sites</t>
   </si>
   <si>
-    <t>DigiKey Alternate</t>
-  </si>
-  <si>
     <t>SLG7NT402V</t>
   </si>
   <si>
@@ -116,6 +101,21 @@
   </si>
   <si>
     <t>Connector</t>
+  </si>
+  <si>
+    <t>Manufacturer Part Number</t>
+  </si>
+  <si>
+    <t>Digikey Alternate</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Component Name</t>
+  </si>
+  <si>
+    <t>S.No</t>
   </si>
 </sst>
 </file>
@@ -173,7 +173,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -183,87 +183,16 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thick">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top style="thick">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </right>
-      <top style="thick">
-        <color theme="0"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top/>
       <bottom style="thin">
-        <color theme="0"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -272,58 +201,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -641,159 +546,159 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA640E7F-E624-464F-B8ED-583DBA0569DC}">
   <dimension ref="A2:H13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.5546875" customWidth="1"/>
+    <col min="3" max="3" width="40.88671875" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="26.140625" customWidth="1"/>
+    <col min="8" max="8" width="34.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="H2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="H3" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>4</v>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>1</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" s="7"/>
     </row>
-    <row r="4" spans="1:8" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
-        <v>2</v>
-      </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="9"/>
-      <c r="G4" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="9"/>
-    </row>
-    <row r="5" spans="1:8" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>3</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
-        <v>4</v>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>5</v>
-      </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-    </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
-        <v>6</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="H8" s="9"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D13" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LED, inverter IC and supervisor IC added.
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Part Selection.xlsx
+++ b/Documents/Dev-Files/Part Selection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24620"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF25AFE-F4FD-48EC-A690-67773A2FFDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E07F85B-87E6-498D-9F55-D3C60D2948B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>Description</t>
   </si>
@@ -116,24 +116,37 @@
   </si>
   <si>
     <t>S.No</t>
+  </si>
+  <si>
+    <t>IC INVERTER OD 1CH 1-INP SC70-5</t>
+  </si>
+  <si>
+    <t>NC7SZ05P5X</t>
+  </si>
+  <si>
+    <t>XC61CN2502MR</t>
+  </si>
+  <si>
+    <t>LED LAMP</t>
+  </si>
+  <si>
+    <t>1W LED</t>
+  </si>
+  <si>
+    <t>-----</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -197,42 +210,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -545,174 +541,307 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA640E7F-E624-464F-B8ED-583DBA0569DC}">
-  <dimension ref="A2:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:H19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
-    <col min="3" max="3" width="40.88671875" customWidth="1"/>
-    <col min="4" max="4" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="3" max="3" width="40.85546875" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="34.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="8" t="s">
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>3</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8" t="s">
+      <c r="F6" s="3"/>
+      <c r="G6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>5</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="7">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8" t="s">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D13" s="1"/>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B3:B10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" xr:uid="{B9773254-489E-4981-AD57-E06C75AC1D1B}"/>
     <hyperlink ref="G3" r:id="rId2" xr:uid="{E9B95C05-B41C-4877-99DA-9D0B95A29B4E}"/>
     <hyperlink ref="G5" r:id="rId3" xr:uid="{2CC3C96D-9B1A-4A63-8F2F-202DB24A48FE}"/>
     <hyperlink ref="G6" r:id="rId4" xr:uid="{7E117F9F-8F90-4E69-A531-92FE100C33C9}"/>
-    <hyperlink ref="G8" r:id="rId5" xr:uid="{0D1B945F-FB9A-413C-807D-F04C4AB6F79F}"/>
+    <hyperlink ref="G12" r:id="rId5" xr:uid="{0D1B945F-FB9A-413C-807D-F04C4AB6F79F}"/>
+    <hyperlink ref="G11" r:id="rId6" xr:uid="{7151ED9F-D159-4F94-87A8-B9212A09D718}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{7F5A0CBF-A840-45D3-A353-B326E51A76B3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ATMEGA, TP5000, power LED, 2 USB connectors and DC jack added to lib.
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Part Selection.xlsx
+++ b/Documents/Dev-Files/Part Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E07F85B-87E6-498D-9F55-D3C60D2948B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD03EDD9-4C29-4889-AB79-DAEC39FA8677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>Description</t>
   </si>
@@ -76,9 +77,6 @@
     <t>DigiKey</t>
   </si>
   <si>
-    <t>DC-C300-5.5A-2.5</t>
-  </si>
-  <si>
     <t>TPS2115ADRBTG4</t>
   </si>
   <si>
@@ -97,9 +95,6 @@
     <t>Ics</t>
   </si>
   <si>
-    <t>5.5A Jack DCPowerReceptacle 6.0mm 2.5mm</t>
-  </si>
-  <si>
     <t>Connector</t>
   </si>
   <si>
@@ -133,17 +128,38 @@
     <t>1W LED</t>
   </si>
   <si>
-    <t>-----</t>
-  </si>
-  <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>901-141A1011D10100</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>USB - Type A 4 USB 2.0 Female 1.5A - USB Connectors ROHS</t>
+  </si>
+  <si>
+    <t>U241-041N-1BR85-1</t>
+  </si>
+  <si>
+    <t>USB - Type B 4 USB 2.0 Female Through Hole USB Connectors ROHS</t>
+  </si>
+  <si>
+    <t>1W 2835 package warm light LED</t>
+  </si>
+  <si>
+    <t>DC-C024E-7A-1.65</t>
+  </si>
+  <si>
+    <t>DC barrel Jack</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +171,21 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -210,10 +241,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -227,8 +259,30 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -554,19 +608,19 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>5</v>
@@ -575,15 +629,15 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>20</v>
+      <c r="B3" s="11" t="s">
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
@@ -595,7 +649,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -606,7 +660,7 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
@@ -617,7 +671,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="H4" s="3"/>
@@ -626,16 +680,16 @@
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
+      <c r="B5" s="11"/>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -646,48 +700,48 @@
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="11"/>
       <c r="C6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="11"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="G7" s="5"/>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="11"/>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="6" t="s">
         <v>2</v>
       </c>
       <c r="H8" s="3"/>
@@ -696,26 +750,26 @@
       <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="11"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="G9" s="5"/>
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="11"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -723,59 +777,79 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
         <v>33</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H11" s="2"/>
+      <c r="G11" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="3"/>
+        <v>38</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="F12" s="3"/>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="6" t="s">
         <v>2</v>
       </c>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="C13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>33</v>
+      </c>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="G13" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+      <c r="C14" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="G14" s="9" t="s">
+        <v>2</v>
+      </c>
       <c r="H14" s="3"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -838,10 +912,12 @@
     <hyperlink ref="G5" r:id="rId3" xr:uid="{2CC3C96D-9B1A-4A63-8F2F-202DB24A48FE}"/>
     <hyperlink ref="G6" r:id="rId4" xr:uid="{7E117F9F-8F90-4E69-A531-92FE100C33C9}"/>
     <hyperlink ref="G12" r:id="rId5" xr:uid="{0D1B945F-FB9A-413C-807D-F04C4AB6F79F}"/>
-    <hyperlink ref="G11" r:id="rId6" xr:uid="{7151ED9F-D159-4F94-87A8-B9212A09D718}"/>
-    <hyperlink ref="G8" r:id="rId7" xr:uid="{7F5A0CBF-A840-45D3-A353-B326E51A76B3}"/>
+    <hyperlink ref="G8" r:id="rId6" xr:uid="{7F5A0CBF-A840-45D3-A353-B326E51A76B3}"/>
+    <hyperlink ref="G13" r:id="rId7" xr:uid="{BEA04E3A-131C-451E-BA13-7E0C4141C71A}"/>
+    <hyperlink ref="G14" r:id="rId8" xr:uid="{7E5F44D1-58EE-4FB2-979F-12617FEF1A85}"/>
+    <hyperlink ref="G11" r:id="rId9" xr:uid="{6FD3F8F2-6544-4482-9E4E-7C343C608D49}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId8"/>
+  <pageSetup orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Schamtic Designing. Changes in library.
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Part Selection.xlsx
+++ b/Documents/Dev-Files/Part Selection.xlsx
@@ -1,32 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark-37\Documents\GitHub\BriacBarthes-PhoneCharger\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD03EDD9-4C29-4889-AB79-DAEC39FA8677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C6BF7A-128C-414A-865B-36504D3BE90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{1C19701A-4E31-4C82-B96B-4DECCE606FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -599,11 +591,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" customWidth="1"/>
+    <col min="3" max="3" width="45.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -817,7 +809,9 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
       <c r="B13" s="2"/>
       <c r="C13" s="8" t="s">
         <v>34</v>
@@ -835,7 +829,9 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
       <c r="B14" s="3"/>
       <c r="C14" s="10" t="s">
         <v>36</v>

</xml_diff>